<commit_message>
fix: improve AdjustToContents accuracy by removing per-glyph advance width rounding (ClosedXML/ClosedXML#2771)
Individual glyph advance widths were rounded to the nearest integer pixel
before summing, causing accumulated rounding errors that made columns too
narrow. Store precise float advance widths instead, letting the final
column width calculation handle rounding at the aggregate level.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/XLibur.Tests/Resource/Examples/ConditionalFormatting/CFDataBar.xlsx
+++ b/XLibur.Tests/Resource/Examples/ConditionalFormatting/CFDataBar.xlsx
@@ -396,7 +396,7 @@
       </x:dataBar>
       <x:extLst>
         <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{440ec55b-d27a-4d05-8949-0494753229d3}</x14:id>
+          <x14:id>{67452155-bbec-427a-8f5b-2e896f384e1b}</x14:id>
         </x:ext>
       </x:extLst>
     </x:cfRule>
@@ -410,7 +410,7 @@
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{440ec55b-d27a-4d05-8949-0494753229d3}">
+          <x14:cfRule type="dataBar" id="{67452155-bbec-427a-8f5b-2e896f384e1b}">
             <x14:dataBar minLength="0" maxLength="100" showValue="0" gradient="1">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>

</xml_diff>

<commit_message>
test: regenerate example reference files after font metric fixes
The font style pass-through and EmSize DPI fixes changed column width
and row height calculations slightly. Regenerated all reference xlsx
files to match the corrected metrics.
</commit_message>
<xml_diff>
--- a/XLibur.Tests/Resource/Examples/ConditionalFormatting/CFDataBar.xlsx
+++ b/XLibur.Tests/Resource/Examples/ConditionalFormatting/CFDataBar.xlsx
@@ -396,7 +396,7 @@
       </x:dataBar>
       <x:extLst>
         <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{67452155-bbec-427a-8f5b-2e896f384e1b}</x14:id>
+          <x14:id>{3cc20586-5dbb-45fc-9f17-8e0cd434b803}</x14:id>
         </x:ext>
       </x:extLst>
     </x:cfRule>
@@ -410,7 +410,7 @@
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{67452155-bbec-427a-8f5b-2e896f384e1b}">
+          <x14:cfRule type="dataBar" id="{3cc20586-5dbb-45fc-9f17-8e0cd434b803}">
             <x14:dataBar minLength="0" maxLength="100" showValue="0" gradient="1">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>

</xml_diff>